<commit_message>
feat(saff-study): publish specification and test suite v1.5
</commit_message>
<xml_diff>
--- a/output/xlsx/ExtracaoViaInterfaceMetrix--GT-.xlsx
+++ b/output/xlsx/ExtracaoViaInterfaceMetrix--GT-.xlsx
@@ -110,7 +110,7 @@
     <t>clock: a cada 10 segundos</t>
   </si>
   <si>
-    <t>SYSTEM verifica se existem diretórios de serial number no formato correto e que foram criados a X ou mais tempo definido na propriedade AUTO_COLLECT_WAIT_TIME no arquivo conf.properties e então: envia as extracoes com essas restricoes para o servidor, transfere essas extrações(somente a pasta de serial number) para a pasta 'AUTO_COLLECT_READ_DIR/PRODUCTNUMBER'(onde o PRODUCTNUMBER é referente a cada SERIALNUMBER), atualiza o contador de extrações realizadas/enviadas e fica em espera por novas extracoes com essas mesmas restricoes na pasta indicada, verifica se existe conexão com o servidor para enviar as extrações offline</t>
+    <t>SYSTEM verifica se existem diretórios de serial number no formato correto e que foram criados a X ou mais tempo definido na propriedade AUTO_COLLECT_WAIT_TIME no arquivo conf.properties e então: envia as extracoes com essas restricoes para o servidor, transfere essas extrações(somente a pasta de serial number) para a pasta 'AUTO_COLLECT_READ_DIR/PRODUCTNUMBER'(onde o PRODUCTNUMBER é referente a cada SERIALNUMBER), atualiza o contador de extrações realizadas/enviadas e fica em espera por novas extracoes com essas mesmas restricoes na pasta indicada</t>
   </si>
   <si>
     <t>administrador: pressiona botao 'Stop'</t>
@@ -128,7 +128,7 @@
     <t>TC2</t>
   </si>
   <si>
-    <t>Alternative Flow 1: Altera a pasta C:\\Collect para uma pasta vazia</t>
+    <t>Alternative Flow 1: Altera a pasta C\:\\Collect para uma pasta vazia</t>
   </si>
   <si>
     <t>administrador: seleciona pasta vazia, e pressiona botao 'Start'</t>

</xml_diff>

<commit_message>
feat(saff-study): publish specification and test suite v2.3
</commit_message>
<xml_diff>
--- a/output/xlsx/ExtracaoViaInterfaceMetrix--GT-.xlsx
+++ b/output/xlsx/ExtracaoViaInterfaceMetrix--GT-.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="50">
   <si>
     <t xml:space="preserve">System: </t>
   </si>
@@ -38,7 +38,7 @@
     <t>Reduced (Greedy Heuristic - Transition Coverage)</t>
   </si>
   <si>
-    <t>Size: 5 test case(s)</t>
+    <t>Size: 4 test case(s)</t>
   </si>
   <si>
     <t xml:space="preserve">Creation Date: </t>
@@ -162,15 +162,6 @@
   </si>
   <si>
     <t>Flow interrupted due to exception / error</t>
-  </si>
-  <si>
-    <t>TC5</t>
-  </si>
-  <si>
-    <t>Exception Flow 2: Extração não se encontra em formato adequado</t>
-  </si>
-  <si>
-    <t>SYSTEM move a extração para a pasta broken</t>
   </si>
 </sst>
 </file>
@@ -262,7 +253,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F60"/>
+  <dimension ref="A1:F50"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="17.578125" customWidth="true" bestFit="true"/>
@@ -936,127 +927,6 @@
         <v>49</v>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" t="s" s="1">
-        <v>11</v>
-      </c>
-      <c r="B53" t="s" s="0">
-        <v>50</v>
-      </c>
-      <c r="C53" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="E53" t="s" s="1">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="s" s="1">
-        <v>15</v>
-      </c>
-      <c r="B54" t="s" s="0">
-        <v>51</v>
-      </c>
-      <c r="E54" t="s" s="1">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="s" s="1">
-        <v>18</v>
-      </c>
-      <c r="B55" t="s" s="0">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="B56" t="s" s="2">
-        <v>21</v>
-      </c>
-      <c r="C56" t="s" s="2">
-        <v>22</v>
-      </c>
-      <c r="D56" t="s" s="2">
-        <v>23</v>
-      </c>
-      <c r="E56" t="s" s="2">
-        <v>24</v>
-      </c>
-      <c r="F56" t="s" s="2">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="n" s="4">
-        <v>1.0</v>
-      </c>
-      <c r="B57" t="s" s="3">
-        <v>26</v>
-      </c>
-      <c r="C57" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D57" t="s" s="3">
-        <v>28</v>
-      </c>
-      <c r="E57" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F57" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="n" s="4">
-        <v>2.0</v>
-      </c>
-      <c r="B58" t="s" s="3">
-        <v>29</v>
-      </c>
-      <c r="C58" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D58" t="s" s="3">
-        <v>30</v>
-      </c>
-      <c r="E58" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F58" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="n" s="4">
-        <v>3.0</v>
-      </c>
-      <c r="B59" t="s" s="3">
-        <v>31</v>
-      </c>
-      <c r="C59" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D59" t="s" s="3">
-        <v>52</v>
-      </c>
-      <c r="E59" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F59" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="s" s="1">
-        <v>35</v>
-      </c>
-      <c r="B60" t="s" s="0">
-        <v>49</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(saff-study): publish specification and test suite v2.5
</commit_message>
<xml_diff>
--- a/output/xlsx/ExtracaoViaInterfaceMetrix--GT-.xlsx
+++ b/output/xlsx/ExtracaoViaInterfaceMetrix--GT-.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="51">
   <si>
     <t xml:space="preserve">System: </t>
   </si>
@@ -110,7 +110,7 @@
     <t>administrador: seleciona uma pasta contendo varias extracoes, seta as informacoes solicitadas na tela inicial e pressiona o botao 'Start'</t>
   </si>
   <si>
-    <t>SYSTEM bloqueia todos os botoes, com excecao do botao 'Stop'</t>
+    <t>SYSTEM processes action successfully</t>
   </si>
   <si>
     <t>clock: a cada 30 segundos</t>
@@ -128,7 +128,7 @@
     <t xml:space="preserve">Postcondition: </t>
   </si>
   <si>
-    <t>As extracoes da pasta indicada devem ter sido enviadas para o servidor e transferidas para a pasta 'read'</t>
+    <t>As extracoes da pasta indicada deve ter sido enviadas para o servidor e transferidas para a pasta 'read'</t>
   </si>
   <si>
     <t>TC2</t>
@@ -141,9 +141,6 @@
   </si>
   <si>
     <t>SYSTEM fica em espera ate que alguma extracao seja adicionada na pasta indicada</t>
-  </si>
-  <si>
-    <t>administrador: adiciona extracao a pasta indicada</t>
   </si>
   <si>
     <t>TC3</t>
@@ -259,7 +256,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F54"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="17.578125" customWidth="true" bestFit="true"/>
@@ -588,13 +585,13 @@
         <v>4.0</v>
       </c>
       <c r="B25" t="s" s="3">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="C25" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D25" t="s" s="3">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E25" t="s" s="3">
         <v>27</v>
@@ -608,13 +605,13 @@
         <v>5.0</v>
       </c>
       <c r="B26" t="s" s="3">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C26" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D26" t="s" s="3">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E26" t="s" s="3">
         <v>27</v>
@@ -624,98 +621,98 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="n" s="4">
-        <v>6.0</v>
-      </c>
-      <c r="B27" t="s" s="3">
-        <v>35</v>
-      </c>
-      <c r="C27" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D27" t="s" s="3">
-        <v>36</v>
-      </c>
-      <c r="E27" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F27" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="s" s="1">
+      <c r="A27" t="s" s="1">
         <v>37</v>
       </c>
-      <c r="B28" t="s" s="0">
+      <c r="B27" t="s" s="0">
         <v>38</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s" s="1">
+        <v>11</v>
+      </c>
+      <c r="B30" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="C30" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="E30" t="s" s="1">
+        <v>14</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s" s="1">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B31" t="s" s="0">
         <v>44</v>
       </c>
-      <c r="C31" t="s" s="1">
-        <v>13</v>
-      </c>
       <c r="E31" t="s" s="1">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s" s="1">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B32" t="s" s="0">
-        <v>45</v>
-      </c>
-      <c r="E32" t="s" s="1">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="s" s="1">
-        <v>18</v>
-      </c>
-      <c r="B33" t="s" s="0">
-        <v>19</v>
+      <c r="A33" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="B33" t="s" s="2">
+        <v>21</v>
+      </c>
+      <c r="C33" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="D33" t="s" s="2">
+        <v>23</v>
+      </c>
+      <c r="E33" t="s" s="2">
+        <v>24</v>
+      </c>
+      <c r="F33" t="s" s="2">
+        <v>25</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="B34" t="s" s="2">
-        <v>21</v>
-      </c>
-      <c r="C34" t="s" s="2">
-        <v>22</v>
-      </c>
-      <c r="D34" t="s" s="2">
-        <v>23</v>
-      </c>
-      <c r="E34" t="s" s="2">
-        <v>24</v>
-      </c>
-      <c r="F34" t="s" s="2">
-        <v>25</v>
+      <c r="A34" t="n" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="B34" t="s" s="3">
+        <v>26</v>
+      </c>
+      <c r="C34" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D34" t="s" s="3">
+        <v>28</v>
+      </c>
+      <c r="E34" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F34" t="s" s="3">
+        <v>27</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n" s="4">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="B35" t="s" s="3">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C35" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D35" t="s" s="3">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E35" t="s" s="3">
         <v>27</v>
@@ -726,16 +723,16 @@
     </row>
     <row r="36">
       <c r="A36" t="n" s="4">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="B36" t="s" s="3">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C36" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D36" t="s" s="3">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E36" t="s" s="3">
         <v>27</v>
@@ -746,10 +743,10 @@
     </row>
     <row r="37">
       <c r="A37" t="n" s="4">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="B37" t="s" s="3">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C37" t="s" s="3">
         <v>27</v>
@@ -766,16 +763,16 @@
     </row>
     <row r="38">
       <c r="A38" t="n" s="4">
-        <v>4.0</v>
+        <v>5.0</v>
       </c>
       <c r="B38" t="s" s="3">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="C38" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D38" t="s" s="3">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E38" t="s" s="3">
         <v>27</v>
@@ -785,138 +782,138 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="n" s="4">
-        <v>5.0</v>
-      </c>
-      <c r="B39" t="s" s="3">
-        <v>46</v>
-      </c>
-      <c r="C39" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D39" t="s" s="3">
-        <v>32</v>
-      </c>
-      <c r="E39" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F39" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="n" s="4">
-        <v>6.0</v>
-      </c>
-      <c r="B40" t="s" s="3">
-        <v>33</v>
-      </c>
-      <c r="C40" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D40" t="s" s="3">
-        <v>34</v>
-      </c>
-      <c r="E40" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F40" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="n" s="4">
-        <v>7.0</v>
-      </c>
-      <c r="B41" t="s" s="3">
-        <v>35</v>
-      </c>
-      <c r="C41" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D41" t="s" s="3">
-        <v>36</v>
-      </c>
-      <c r="E41" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F41" t="s" s="3">
-        <v>27</v>
+      <c r="A39" t="s" s="1">
+        <v>37</v>
+      </c>
+      <c r="B39" t="s" s="0">
+        <v>38</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="1">
-        <v>37</v>
+        <v>11</v>
       </c>
       <c r="B42" t="s" s="0">
-        <v>38</v>
+        <v>46</v>
+      </c>
+      <c r="C42" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="E42" t="s" s="1">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="B43" t="s" s="0">
+        <v>47</v>
+      </c>
+      <c r="E43" t="s" s="1">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="s" s="1">
+        <v>18</v>
+      </c>
+      <c r="B44" t="s" s="0">
+        <v>19</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="s" s="1">
-        <v>11</v>
-      </c>
-      <c r="B45" t="s" s="0">
-        <v>47</v>
-      </c>
-      <c r="C45" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="E45" t="s" s="1">
-        <v>14</v>
+      <c r="A45" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="B45" t="s" s="2">
+        <v>21</v>
+      </c>
+      <c r="C45" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="D45" t="s" s="2">
+        <v>23</v>
+      </c>
+      <c r="E45" t="s" s="2">
+        <v>24</v>
+      </c>
+      <c r="F45" t="s" s="2">
+        <v>25</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="s" s="1">
-        <v>15</v>
-      </c>
-      <c r="B46" t="s" s="0">
-        <v>48</v>
-      </c>
-      <c r="E46" t="s" s="1">
-        <v>17</v>
+      <c r="A46" t="n" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="B46" t="s" s="3">
+        <v>26</v>
+      </c>
+      <c r="C46" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D46" t="s" s="3">
+        <v>28</v>
+      </c>
+      <c r="E46" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F46" t="s" s="3">
+        <v>27</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="s" s="1">
-        <v>18</v>
-      </c>
-      <c r="B47" t="s" s="0">
-        <v>19</v>
+      <c r="A47" t="n" s="4">
+        <v>2.0</v>
+      </c>
+      <c r="B47" t="s" s="3">
+        <v>29</v>
+      </c>
+      <c r="C47" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D47" t="s" s="3">
+        <v>30</v>
+      </c>
+      <c r="E47" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F47" t="s" s="3">
+        <v>27</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="B48" t="s" s="2">
-        <v>21</v>
-      </c>
-      <c r="C48" t="s" s="2">
-        <v>22</v>
-      </c>
-      <c r="D48" t="s" s="2">
-        <v>23</v>
-      </c>
-      <c r="E48" t="s" s="2">
-        <v>24</v>
-      </c>
-      <c r="F48" t="s" s="2">
-        <v>25</v>
+      <c r="A48" t="n" s="4">
+        <v>3.0</v>
+      </c>
+      <c r="B48" t="s" s="3">
+        <v>31</v>
+      </c>
+      <c r="C48" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D48" t="s" s="3">
+        <v>32</v>
+      </c>
+      <c r="E48" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F48" t="s" s="3">
+        <v>27</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n" s="4">
-        <v>1.0</v>
+        <v>4.0</v>
       </c>
       <c r="B49" t="s" s="3">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="C49" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D49" t="s" s="3">
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="E49" t="s" s="3">
         <v>27</v>
@@ -927,16 +924,16 @@
     </row>
     <row r="50">
       <c r="A50" t="n" s="4">
-        <v>2.0</v>
+        <v>5.0</v>
       </c>
       <c r="B50" t="s" s="3">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C50" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D50" t="s" s="3">
-        <v>30</v>
+        <v>49</v>
       </c>
       <c r="E50" t="s" s="3">
         <v>27</v>
@@ -946,71 +943,11 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="n" s="4">
-        <v>3.0</v>
-      </c>
-      <c r="B51" t="s" s="3">
-        <v>31</v>
-      </c>
-      <c r="C51" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D51" t="s" s="3">
-        <v>32</v>
-      </c>
-      <c r="E51" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F51" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="n" s="4">
-        <v>4.0</v>
-      </c>
-      <c r="B52" t="s" s="3">
-        <v>33</v>
-      </c>
-      <c r="C52" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D52" t="s" s="3">
-        <v>49</v>
-      </c>
-      <c r="E52" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F52" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="n" s="4">
-        <v>5.0</v>
-      </c>
-      <c r="B53" t="s" s="3">
-        <v>33</v>
-      </c>
-      <c r="C53" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D53" t="s" s="3">
+      <c r="A51" t="s" s="1">
+        <v>37</v>
+      </c>
+      <c r="B51" t="s" s="0">
         <v>50</v>
-      </c>
-      <c r="E53" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F53" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="s" s="1">
-        <v>37</v>
-      </c>
-      <c r="B54" t="s" s="0">
-        <v>51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(saff-study): publish specification and test suite v2.6
</commit_message>
<xml_diff>
--- a/output/xlsx/ExtracaoViaInterfaceMetrix--GT-.xlsx
+++ b/output/xlsx/ExtracaoViaInterfaceMetrix--GT-.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="51">
   <si>
     <t xml:space="preserve">System: </t>
   </si>
@@ -71,7 +71,7 @@
     <t xml:space="preserve">Precondition: </t>
   </si>
   <si>
-    <t>Usuario deve estar logado como administrador</t>
+    <t>Usuário deve estar logado no servidor e no extrator como administrador</t>
   </si>
   <si>
     <t>#</t>
@@ -92,63 +92,63 @@
     <t>Actual Result</t>
   </si>
   <si>
-    <t>administrador: configura o extrator para iniciar em modo 'Automatic Collection'</t>
+    <t>administrador: seta o extrator para iniciar em modo 'Automatic Collection' e faz login no extrator</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>SYSTEM exibe tela de login</t>
-  </si>
-  <si>
-    <t>administrador: faz login no extrator</t>
-  </si>
-  <si>
-    <t>SYSTEM exibe tela de coleta automatica</t>
-  </si>
-  <si>
-    <t>administrador: seleciona uma pasta contendo varias extracoes, seta as informacoes solicitadas na tela inicial e pressiona o botao 'Start'</t>
+    <t>SYSTEM exibe tela inicial do extrator</t>
+  </si>
+  <si>
+    <t>administrador: seleciona pasta contendo varias extracoes, seta as informacoes solicitadas na tela inicial e pressiona o botão 'Start'</t>
+  </si>
+  <si>
+    <t>SYSTEM renomeia e transfere extracoes para uma pasta temporaria; atualiza contador de extracoes realizadas; demais botoes estao todos bloqueados, com excecao do botao 'Stop'</t>
+  </si>
+  <si>
+    <t>clock: a cada 30 segundos</t>
+  </si>
+  <si>
+    <t>SYSTEM envia extracoes da pasta temporaria para o servidor e fica em espera por novas extracoes na pasta indicada</t>
+  </si>
+  <si>
+    <t>administrador: pressiona botao 'Stop'</t>
+  </si>
+  <si>
+    <t>SYSTEM retorna para tela incial</t>
+  </si>
+  <si>
+    <t>administrador: vai para pagina de visualizacao de extracoes no servidor</t>
+  </si>
+  <si>
+    <t>SYSTEM exibe tela de visualização de extracoes com extracoes recentes no topo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Postcondition: </t>
+  </si>
+  <si>
+    <t>TC2</t>
+  </si>
+  <si>
+    <t>Alternative Flow 1: Seleciona pasta vazia</t>
+  </si>
+  <si>
+    <t>administrador: seleciona pasta vazia, e pressiona botão 'Start'</t>
+  </si>
+  <si>
+    <t>SYSTEM fica em espera ate que usuario insira alguma extracao na pasta indicada</t>
+  </si>
+  <si>
+    <t>TC3</t>
+  </si>
+  <si>
+    <t>Alternative Flow 2: Insere novas extracoes na pasta</t>
   </si>
   <si>
     <t>SYSTEM processes action successfully</t>
   </si>
   <si>
-    <t>clock: a cada 30 segundos</t>
-  </si>
-  <si>
-    <t>SYSTEM envia extracoes para o servidor, transfere essas extrações para a pasta 'read', atualiza o contador de extrações realizadas e fica em espera por novas extracoes na pasta indicada</t>
-  </si>
-  <si>
-    <t>administrador: pressiona botao 'Stop'</t>
-  </si>
-  <si>
-    <t>SYSTEM desbloqueia todos os botoes e para de escutar a pasta indicada</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Postcondition: </t>
-  </si>
-  <si>
-    <t>As extracoes da pasta indicada deve ter sido enviadas para o servidor e transferidas para a pasta 'read'</t>
-  </si>
-  <si>
-    <t>TC2</t>
-  </si>
-  <si>
-    <t>Alternative Flow 1: Seleciona pasta vazia</t>
-  </si>
-  <si>
-    <t>administrador: seleciona pasta vazia, e pressiona botao 'Start'</t>
-  </si>
-  <si>
-    <t>SYSTEM fica em espera ate que alguma extracao seja adicionada na pasta indicada</t>
-  </si>
-  <si>
-    <t>TC3</t>
-  </si>
-  <si>
-    <t>Alternative Flow 2: Insere novas extracoes na pasta</t>
-  </si>
-  <si>
     <t>administrador: adiciona novas extracoes na pasta indicada</t>
   </si>
   <si>
@@ -158,10 +158,10 @@
     <t>Exception Flow 1: Falha no envio ao servidor</t>
   </si>
   <si>
-    <t>SYSTEM mantem a informacao de quais extracoes foram enviadas para o servidor; fica em espera ate que a conexao seja reestabelecida</t>
-  </si>
-  <si>
-    <t>SYSTEM tenta enviar extrações restantes para o servidor</t>
+    <t>SYSTEM mantem informacao de quais extracoes foram enviadas; fica em espera ate que a conexao seja reestabelecida</t>
+  </si>
+  <si>
+    <t>SYSTEM tenta enviar extracoes restantes para o servidor</t>
   </si>
   <si>
     <t>Flow interrupted due to exception / error</t>
@@ -256,13 +256,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="17.578125" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="109.10546875" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="105.1015625" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="21.8984375" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="149.2421875" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="145.60546875" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="30.5234375" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="17.578125" customWidth="true" bestFit="true"/>
   </cols>
@@ -464,7 +464,7 @@
         <v>37</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>38</v>
+        <v>27</v>
       </c>
     </row>
     <row r="18">
@@ -472,7 +472,7 @@
         <v>11</v>
       </c>
       <c r="B18" t="s" s="0">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C18" t="s" s="1">
         <v>13</v>
@@ -486,7 +486,7 @@
         <v>15</v>
       </c>
       <c r="B19" t="s" s="0">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E19" t="s" s="1">
         <v>17</v>
@@ -545,13 +545,13 @@
         <v>2.0</v>
       </c>
       <c r="B23" t="s" s="3">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="C23" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D23" t="s" s="3">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="E23" t="s" s="3">
         <v>27</v>
@@ -561,138 +561,138 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="n" s="4">
-        <v>3.0</v>
-      </c>
-      <c r="B24" t="s" s="3">
-        <v>41</v>
-      </c>
-      <c r="C24" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D24" t="s" s="3">
-        <v>42</v>
-      </c>
-      <c r="E24" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F24" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="n" s="4">
-        <v>4.0</v>
-      </c>
-      <c r="B25" t="s" s="3">
-        <v>33</v>
-      </c>
-      <c r="C25" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D25" t="s" s="3">
-        <v>34</v>
-      </c>
-      <c r="E25" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F25" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="n" s="4">
-        <v>5.0</v>
-      </c>
-      <c r="B26" t="s" s="3">
-        <v>35</v>
-      </c>
-      <c r="C26" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D26" t="s" s="3">
-        <v>36</v>
-      </c>
-      <c r="E26" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F26" t="s" s="3">
+      <c r="A24" t="s" s="1">
+        <v>37</v>
+      </c>
+      <c r="B24" t="s" s="0">
         <v>27</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s" s="1">
-        <v>37</v>
+        <v>11</v>
       </c>
       <c r="B27" t="s" s="0">
-        <v>38</v>
+        <v>42</v>
+      </c>
+      <c r="C27" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="E27" t="s" s="1">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="B28" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="E28" t="s" s="1">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s" s="1">
+        <v>18</v>
+      </c>
+      <c r="B29" t="s" s="0">
+        <v>19</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="s" s="1">
-        <v>11</v>
-      </c>
-      <c r="B30" t="s" s="0">
-        <v>43</v>
-      </c>
-      <c r="C30" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="E30" t="s" s="1">
-        <v>14</v>
+      <c r="A30" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="B30" t="s" s="2">
+        <v>21</v>
+      </c>
+      <c r="C30" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="D30" t="s" s="2">
+        <v>23</v>
+      </c>
+      <c r="E30" t="s" s="2">
+        <v>24</v>
+      </c>
+      <c r="F30" t="s" s="2">
+        <v>25</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="s" s="1">
-        <v>15</v>
-      </c>
-      <c r="B31" t="s" s="0">
+      <c r="A31" t="n" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="B31" t="s" s="3">
+        <v>26</v>
+      </c>
+      <c r="C31" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D31" t="s" s="3">
+        <v>28</v>
+      </c>
+      <c r="E31" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F31" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n" s="4">
+        <v>2.0</v>
+      </c>
+      <c r="B32" t="s" s="3">
+        <v>29</v>
+      </c>
+      <c r="C32" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D32" t="s" s="3">
+        <v>30</v>
+      </c>
+      <c r="E32" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F32" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n" s="4">
+        <v>3.0</v>
+      </c>
+      <c r="B33" t="s" s="3">
+        <v>31</v>
+      </c>
+      <c r="C33" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D33" t="s" s="3">
         <v>44</v>
       </c>
-      <c r="E31" t="s" s="1">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="s" s="1">
-        <v>18</v>
-      </c>
-      <c r="B32" t="s" s="0">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="B33" t="s" s="2">
-        <v>21</v>
-      </c>
-      <c r="C33" t="s" s="2">
-        <v>22</v>
-      </c>
-      <c r="D33" t="s" s="2">
-        <v>23</v>
-      </c>
-      <c r="E33" t="s" s="2">
-        <v>24</v>
-      </c>
-      <c r="F33" t="s" s="2">
-        <v>25</v>
+      <c r="E33" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F33" t="s" s="3">
+        <v>27</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n" s="4">
-        <v>1.0</v>
+        <v>4.0</v>
       </c>
       <c r="B34" t="s" s="3">
-        <v>26</v>
+        <v>45</v>
       </c>
       <c r="C34" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D34" t="s" s="3">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E34" t="s" s="3">
         <v>27</v>
@@ -703,16 +703,16 @@
     </row>
     <row r="35">
       <c r="A35" t="n" s="4">
-        <v>2.0</v>
+        <v>5.0</v>
       </c>
       <c r="B35" t="s" s="3">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C35" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D35" t="s" s="3">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E35" t="s" s="3">
         <v>27</v>
@@ -723,16 +723,16 @@
     </row>
     <row r="36">
       <c r="A36" t="n" s="4">
-        <v>3.0</v>
+        <v>6.0</v>
       </c>
       <c r="B36" t="s" s="3">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C36" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D36" t="s" s="3">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E36" t="s" s="3">
         <v>27</v>
@@ -743,16 +743,16 @@
     </row>
     <row r="37">
       <c r="A37" t="n" s="4">
-        <v>4.0</v>
+        <v>7.0</v>
       </c>
       <c r="B37" t="s" s="3">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C37" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D37" t="s" s="3">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="E37" t="s" s="3">
         <v>27</v>
@@ -762,98 +762,98 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="n" s="4">
-        <v>5.0</v>
-      </c>
-      <c r="B38" t="s" s="3">
-        <v>45</v>
-      </c>
-      <c r="C38" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D38" t="s" s="3">
-        <v>32</v>
-      </c>
-      <c r="E38" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F38" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="s" s="1">
+      <c r="A38" t="s" s="1">
         <v>37</v>
       </c>
-      <c r="B39" t="s" s="0">
-        <v>38</v>
+      <c r="B38" t="s" s="0">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="s" s="1">
+        <v>11</v>
+      </c>
+      <c r="B41" t="s" s="0">
+        <v>46</v>
+      </c>
+      <c r="C41" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="E41" t="s" s="1">
+        <v>14</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="1">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B42" t="s" s="0">
-        <v>46</v>
-      </c>
-      <c r="C42" t="s" s="1">
-        <v>13</v>
+        <v>47</v>
       </c>
       <c r="E42" t="s" s="1">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s" s="1">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B43" t="s" s="0">
-        <v>47</v>
-      </c>
-      <c r="E43" t="s" s="1">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="s" s="1">
-        <v>18</v>
-      </c>
-      <c r="B44" t="s" s="0">
-        <v>19</v>
+      <c r="A44" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="B44" t="s" s="2">
+        <v>21</v>
+      </c>
+      <c r="C44" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="D44" t="s" s="2">
+        <v>23</v>
+      </c>
+      <c r="E44" t="s" s="2">
+        <v>24</v>
+      </c>
+      <c r="F44" t="s" s="2">
+        <v>25</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="B45" t="s" s="2">
-        <v>21</v>
-      </c>
-      <c r="C45" t="s" s="2">
-        <v>22</v>
-      </c>
-      <c r="D45" t="s" s="2">
-        <v>23</v>
-      </c>
-      <c r="E45" t="s" s="2">
-        <v>24</v>
-      </c>
-      <c r="F45" t="s" s="2">
-        <v>25</v>
+      <c r="A45" t="n" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="B45" t="s" s="3">
+        <v>26</v>
+      </c>
+      <c r="C45" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D45" t="s" s="3">
+        <v>28</v>
+      </c>
+      <c r="E45" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F45" t="s" s="3">
+        <v>27</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n" s="4">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="B46" t="s" s="3">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C46" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D46" t="s" s="3">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E46" t="s" s="3">
         <v>27</v>
@@ -864,16 +864,16 @@
     </row>
     <row r="47">
       <c r="A47" t="n" s="4">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="B47" t="s" s="3">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C47" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D47" t="s" s="3">
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="E47" t="s" s="3">
         <v>27</v>
@@ -884,7 +884,7 @@
     </row>
     <row r="48">
       <c r="A48" t="n" s="4">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="B48" t="s" s="3">
         <v>31</v>
@@ -893,7 +893,7 @@
         <v>27</v>
       </c>
       <c r="D48" t="s" s="3">
-        <v>32</v>
+        <v>49</v>
       </c>
       <c r="E48" t="s" s="3">
         <v>27</v>
@@ -903,50 +903,10 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="n" s="4">
-        <v>4.0</v>
-      </c>
-      <c r="B49" t="s" s="3">
-        <v>33</v>
-      </c>
-      <c r="C49" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D49" t="s" s="3">
-        <v>48</v>
-      </c>
-      <c r="E49" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F49" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="n" s="4">
-        <v>5.0</v>
-      </c>
-      <c r="B50" t="s" s="3">
-        <v>33</v>
-      </c>
-      <c r="C50" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D50" t="s" s="3">
-        <v>49</v>
-      </c>
-      <c r="E50" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F50" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="s" s="1">
+      <c r="A49" t="s" s="1">
         <v>37</v>
       </c>
-      <c r="B51" t="s" s="0">
+      <c r="B49" t="s" s="0">
         <v>50</v>
       </c>
     </row>

</xml_diff>